<commit_message>
Start to better describe head of the notebook
Simultaneously with the writing of the user manual
</commit_message>
<xml_diff>
--- a/Feed_optimization/DE_optim_feval_20.11.2025_diet.xlsx
+++ b/Feed_optimization/DE_optim_feval_20.11.2025_diet.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polimi365-my.sharepoint.com/personal/10530006_polimi_it/Documents/Work_cloud/DOTTORATO/Modelling/Pilot_plant/Feed_optimization/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_5F53833861E9913700FE31D2F8F2D3C2445B5DFC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E55851B5-59DB-4708-A958-8472BCF60DAD}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -43,8 +49,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -103,17 +109,25 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -151,7 +165,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -185,6 +199,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -219,9 +234,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -394,11 +410,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H88"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -424,9 +440,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>10.99999999999999</v>
+        <v>10.999999999999989</v>
       </c>
       <c r="B2">
         <v>-42</v>
@@ -435,7 +451,7 @@
         <v>24</v>
       </c>
       <c r="D2">
-        <v>0.9113743622080462</v>
+        <v>0.91137436220804624</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -447,36 +463,36 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>0.9113743622080462</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
+        <v>0.91137436220804624</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>163.4021522207253</v>
       </c>
       <c r="B3">
-        <v>52.70840637064757</v>
+        <v>52.708406370647573</v>
       </c>
       <c r="C3">
-        <v>81.63158688324658</v>
+        <v>81.631586883246584</v>
       </c>
       <c r="D3">
-        <v>0.9629761123779557</v>
+        <v>0.96297611237795566</v>
       </c>
       <c r="E3">
-        <v>259.3040895234316</v>
+        <v>259.30408952343163</v>
       </c>
       <c r="F3">
-        <v>7.194707258299267E+20</v>
+        <v>7.1947072582992672E+20</v>
       </c>
       <c r="G3">
-        <v>12.65818875418963</v>
+        <v>12.658188754189631</v>
       </c>
       <c r="H3">
-        <v>7.194707258299267E+20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
+        <v>7.1947072582992672E+20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>119.8371767122883</v>
       </c>
@@ -484,13 +500,13 @@
         <v>-14.86279893131754</v>
       </c>
       <c r="C4">
-        <v>72.89759399750683</v>
+        <v>72.897593997506831</v>
       </c>
       <c r="D4">
-        <v>0.9614925521976048</v>
+        <v>0.96149255219760477</v>
       </c>
       <c r="E4">
-        <v>282.5955024605154</v>
+        <v>282.59550246051538</v>
       </c>
       <c r="F4">
         <v>2.567559895197741E+21</v>
@@ -502,44 +518,44 @@
         <v>2.567559895197741E+21</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>186.3131012969558</v>
+        <v>186.31310129695581</v>
       </c>
       <c r="B5">
-        <v>0.4660181440162572</v>
+        <v>0.46601814401625719</v>
       </c>
       <c r="C5">
-        <v>26.55279593962367</v>
+        <v>26.552795939623671</v>
       </c>
       <c r="D5">
-        <v>0.9593782005272183</v>
+        <v>0.95937820052721834</v>
       </c>
       <c r="E5">
-        <v>108.0242007019422</v>
+        <v>108.02420070194221</v>
       </c>
       <c r="F5">
-        <v>1.53676823783898E+17</v>
+        <v>1.5367682378389798E+17</v>
       </c>
       <c r="G5">
         <v>0</v>
       </c>
       <c r="H5">
-        <v>1.536768237838981E+17</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
+        <v>1.5367682378389811E+17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>-86.19768614528532</v>
+        <v>-86.197686145285317</v>
       </c>
       <c r="B6">
-        <v>65.75550703813617</v>
+        <v>65.755507038136173</v>
       </c>
       <c r="C6">
-        <v>-0.7662096251239303</v>
+        <v>-0.76620962512393032</v>
       </c>
       <c r="D6">
-        <v>0.9345092875320009</v>
+        <v>0.93450928753200091</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -551,21 +567,21 @@
         <v>0</v>
       </c>
       <c r="H6">
-        <v>0.9345092875320009</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8">
+        <v>0.93450928753200091</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>-74.82429104730808</v>
       </c>
       <c r="B7">
-        <v>47.11758284091621</v>
+        <v>47.117582840916207</v>
       </c>
       <c r="C7">
         <v>31.23163444861887</v>
       </c>
       <c r="D7">
-        <v>0.9162992232908297</v>
+        <v>0.91629922329082969</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -577,47 +593,47 @@
         <v>0</v>
       </c>
       <c r="H7">
-        <v>0.9162992232908297</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
+        <v>0.91629922329082969</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>155.76475253687</v>
+        <v>155.76475253686999</v>
       </c>
       <c r="B8">
         <v>-40.58191545417894</v>
       </c>
       <c r="C8">
-        <v>20.01751859875017</v>
+        <v>20.017518598750168</v>
       </c>
       <c r="D8">
-        <v>0.9567395076152546</v>
+        <v>0.95673950761525461</v>
       </c>
       <c r="E8">
-        <v>97.12546589229598</v>
+        <v>97.125465892295978</v>
       </c>
       <c r="F8">
-        <v>5.270579632704501E+16</v>
+        <v>5.2705796327045008E+16</v>
       </c>
       <c r="G8">
         <v>0</v>
       </c>
       <c r="H8">
-        <v>5.27057963270451E+16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
+        <v>5.2705796327045104E+16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>-55.78279368263011</v>
+        <v>-55.782793682630107</v>
       </c>
       <c r="B9">
-        <v>-64.35051589778651</v>
+        <v>-64.350515897786508</v>
       </c>
       <c r="C9">
-        <v>62.00976133446851</v>
+        <v>62.009761334468507</v>
       </c>
       <c r="D9">
-        <v>0.9421146949029925</v>
+        <v>0.94211469490299249</v>
       </c>
       <c r="E9">
         <v>160.4644449847963</v>
@@ -632,44 +648,44 @@
         <v>1.269443750571631E+17</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>3.290614799537228</v>
+        <v>3.2906147995372281</v>
       </c>
       <c r="B10">
-        <v>-7.833215800789361</v>
+        <v>-7.8332158007893611</v>
       </c>
       <c r="C10">
-        <v>51.70426132469103</v>
+        <v>51.704261324691032</v>
       </c>
       <c r="D10">
-        <v>0.9523938550776229</v>
+        <v>0.95239385507762286</v>
       </c>
       <c r="E10">
-        <v>145.8688162937545</v>
+        <v>145.86881629375449</v>
       </c>
       <c r="F10">
-        <v>4.257758050217425E+17</v>
+        <v>4.2577580502174253E+17</v>
       </c>
       <c r="G10">
         <v>0</v>
       </c>
       <c r="H10">
-        <v>4.257758050217427E+17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
+        <v>4.2577580502174272E+17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>-9.855481836430602</v>
+        <v>-9.8554818364306023</v>
       </c>
       <c r="B11">
-        <v>-79.135912180913</v>
+        <v>-79.135912180912996</v>
       </c>
       <c r="C11">
-        <v>-19.57182869874581</v>
+        <v>-19.571828698745811</v>
       </c>
       <c r="D11">
-        <v>0.9381060256632233</v>
+        <v>0.93810602566322332</v>
       </c>
       <c r="E11">
         <v>0</v>
@@ -678,24 +694,24 @@
         <v>0</v>
       </c>
       <c r="G11">
-        <v>12.43896058800101</v>
+        <v>12.438960588001009</v>
       </c>
       <c r="H11">
         <v>13.37706661366424</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>8.998963658151022</v>
+        <v>8.9989636581510215</v>
       </c>
       <c r="B12">
-        <v>37.41941518534683</v>
+        <v>37.419415185346828</v>
       </c>
       <c r="C12">
         <v>-4.450979240034818</v>
       </c>
       <c r="D12">
-        <v>0.9252945451911013</v>
+        <v>0.92529454519110133</v>
       </c>
       <c r="E12">
         <v>0</v>
@@ -707,21 +723,21 @@
         <v>0</v>
       </c>
       <c r="H12">
-        <v>0.9252945451911013</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
+        <v>0.92529454519110133</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>-42.06096171889582</v>
+        <v>-42.060961718895818</v>
       </c>
       <c r="B13">
-        <v>-30.55312971978453</v>
+        <v>-30.553129719784529</v>
       </c>
       <c r="C13">
         <v>25.6192528349786</v>
       </c>
       <c r="D13">
-        <v>0.9165783045425914</v>
+        <v>0.91657830454259137</v>
       </c>
       <c r="E13">
         <v>0</v>
@@ -733,73 +749,73 @@
         <v>0</v>
       </c>
       <c r="H13">
-        <v>0.9165783045425914</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
+        <v>0.91657830454259137</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>-17.25368626329218</v>
+        <v>-17.253686263292181</v>
       </c>
       <c r="B14">
-        <v>-45.36360340834702</v>
+        <v>-45.363603408347018</v>
       </c>
       <c r="C14">
-        <v>75.54336847712315</v>
+        <v>75.543368477123153</v>
       </c>
       <c r="D14">
-        <v>0.9564992295271824</v>
+        <v>0.95649922952718236</v>
       </c>
       <c r="E14">
-        <v>311.7575199132218</v>
+        <v>311.75751991322181</v>
       </c>
       <c r="F14">
-        <v>2.54450698936407E+21</v>
+        <v>2.5445069893640698E+21</v>
       </c>
       <c r="G14">
         <v>0</v>
       </c>
       <c r="H14">
-        <v>2.54450698936407E+21</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
+        <v>2.5445069893640698E+21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>128.9910746491593</v>
+        <v>128.99107464915929</v>
       </c>
       <c r="B15">
-        <v>81.68631743605252</v>
+        <v>81.686317436052519</v>
       </c>
       <c r="C15">
-        <v>58.8722268261146</v>
+        <v>58.872226826114598</v>
       </c>
       <c r="D15">
-        <v>0.9609427246784086</v>
+        <v>0.96094272467840858</v>
       </c>
       <c r="E15">
-        <v>158.3089626728944</v>
+        <v>158.30896267289441</v>
       </c>
       <c r="F15">
         <v>2.79069156208898E+18</v>
       </c>
       <c r="G15">
-        <v>8.004055872544702</v>
+        <v>8.0040558725447024</v>
       </c>
       <c r="H15">
         <v>2.79069156208898E+18</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>79.3506819029204</v>
       </c>
       <c r="B16">
-        <v>25.77709454342549</v>
+        <v>25.777094543425491</v>
       </c>
       <c r="C16">
         <v>1.174664876085121</v>
       </c>
       <c r="D16">
-        <v>0.9145435167927367</v>
+        <v>0.91454351679273671</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -811,12 +827,12 @@
         <v>0</v>
       </c>
       <c r="H16">
-        <v>0.9145435167927367</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8">
+        <v>0.91454351679273671</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>65.25517321771591</v>
+        <v>65.255173217715907</v>
       </c>
       <c r="B17">
         <v>15.61455549272608</v>
@@ -825,39 +841,39 @@
         <v>96.8889931136097</v>
       </c>
       <c r="D17">
-        <v>0.9619514044676912</v>
+        <v>0.96195140446769123</v>
       </c>
       <c r="E17">
-        <v>390.5484653751608</v>
+        <v>390.54846537516079</v>
       </c>
       <c r="F17">
-        <v>6.704971501763202E+22</v>
+        <v>6.7049715017632016E+22</v>
       </c>
       <c r="G17">
         <v>0</v>
       </c>
       <c r="H17">
-        <v>6.704971501763202E+22</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8">
+        <v>6.7049715017632016E+22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>172.4354721621367</v>
       </c>
       <c r="B18">
-        <v>-52.98248213987991</v>
+        <v>-52.982482139879913</v>
       </c>
       <c r="C18">
-        <v>-13.1303192350975</v>
+        <v>-13.130319235097501</v>
       </c>
       <c r="D18">
-        <v>0.9441475490847153</v>
+        <v>0.94414754908471532</v>
       </c>
       <c r="E18">
-        <v>20.46720053629748</v>
+        <v>20.467200536297479</v>
       </c>
       <c r="F18">
-        <v>977920959443.1301</v>
+        <v>977920959443.13013</v>
       </c>
       <c r="G18">
         <v>0</v>
@@ -866,18 +882,18 @@
         <v>977920959464.5415</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>26.82312660851918</v>
+        <v>26.823126608519178</v>
       </c>
       <c r="B19">
-        <v>6.451060058636823</v>
+        <v>6.4510600586368234</v>
       </c>
       <c r="C19">
-        <v>-9.010726075973121</v>
+        <v>-9.0107260759731211</v>
       </c>
       <c r="D19">
-        <v>0.9261006475350064</v>
+        <v>0.92610064753500643</v>
       </c>
       <c r="E19">
         <v>0</v>
@@ -889,47 +905,47 @@
         <v>0</v>
       </c>
       <c r="H19">
-        <v>0.9261006475350064</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8">
+        <v>0.92610064753500643</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>48.89408446979029</v>
+        <v>48.894084469790293</v>
       </c>
       <c r="B20">
-        <v>-59.74695294761499</v>
+        <v>-59.746952947614993</v>
       </c>
       <c r="C20">
-        <v>85.20052982185842</v>
+        <v>85.200529821858424</v>
       </c>
       <c r="D20">
-        <v>0.9604758821521702</v>
+        <v>0.96047588215217017</v>
       </c>
       <c r="E20">
-        <v>425.1691187510555</v>
+        <v>425.16911875105552</v>
       </c>
       <c r="F20">
-        <v>2.666911217317909E+23</v>
+        <v>2.6669112173179091E+23</v>
       </c>
       <c r="G20">
         <v>0</v>
       </c>
       <c r="H20">
-        <v>2.666911217317909E+23</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8">
+        <v>2.6669112173179091E+23</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>87.75164815656777</v>
+        <v>87.751648156567768</v>
       </c>
       <c r="B21">
-        <v>73.19909988402043</v>
+        <v>73.199099884020427</v>
       </c>
       <c r="C21">
         <v>36.66198641456387</v>
       </c>
       <c r="D21">
-        <v>0.9566586296921453</v>
+        <v>0.95665862969214532</v>
       </c>
       <c r="E21">
         <v>94.18057122573056</v>
@@ -944,12 +960,12 @@
         <v>1.435909268064169E+16</v>
       </c>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>100.9352849612794</v>
+        <v>100.93528496127939</v>
       </c>
       <c r="B22">
-        <v>-70.8197111991859</v>
+        <v>-70.819711199185903</v>
       </c>
       <c r="C22">
         <v>41.51091874784403</v>
@@ -961,27 +977,27 @@
         <v>171.0881032625484</v>
       </c>
       <c r="F22">
-        <v>1.017649216649827E+19</v>
+        <v>1.0176492166498269E+19</v>
       </c>
       <c r="G22">
         <v>0</v>
       </c>
       <c r="H22">
-        <v>1.017649216649827E+19</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8">
+        <v>1.0176492166498269E+19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>-78.41866092975312</v>
+        <v>-78.418660929753116</v>
       </c>
       <c r="B23">
-        <v>-21.76234123526426</v>
+        <v>-21.762341235264259</v>
       </c>
       <c r="C23">
-        <v>55.18316589736319</v>
+        <v>55.183165897363189</v>
       </c>
       <c r="D23">
-        <v>0.9051112949250035</v>
+        <v>0.90511129492500353</v>
       </c>
       <c r="E23">
         <v>0</v>
@@ -993,24 +1009,24 @@
         <v>0</v>
       </c>
       <c r="H23">
-        <v>0.9051112949250035</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8">
+        <v>0.90511129492500353</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>147.557720340922</v>
       </c>
       <c r="B24">
-        <v>61.5917849770295</v>
+        <v>61.591784977029498</v>
       </c>
       <c r="C24">
-        <v>17.32143581736595</v>
+        <v>17.321435817365948</v>
       </c>
       <c r="D24">
-        <v>0.9566014959662266</v>
+        <v>0.95660149596622657</v>
       </c>
       <c r="E24">
-        <v>65.305934998192</v>
+        <v>65.305934998192001</v>
       </c>
       <c r="F24">
         <v>1151710344919712</v>
@@ -1022,18 +1038,18 @@
         <v>1151710344919778</v>
       </c>
     </row>
-    <row r="25" spans="1:8">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>-47.31107251820578</v>
+        <v>-47.311072518205783</v>
       </c>
       <c r="B25">
-        <v>-33.96776612868369</v>
+        <v>-33.967766128683692</v>
       </c>
       <c r="C25">
-        <v>-28.04525525150433</v>
+        <v>-28.045255251504329</v>
       </c>
       <c r="D25">
-        <v>0.9466981504307181</v>
+        <v>0.94669815043071814</v>
       </c>
       <c r="E25">
         <v>0</v>
@@ -1042,128 +1058,128 @@
         <v>0</v>
       </c>
       <c r="G25">
-        <v>12.83229198018883</v>
+        <v>12.832291980188829</v>
       </c>
       <c r="H25">
         <v>13.77899013061954</v>
       </c>
     </row>
-    <row r="26" spans="1:8">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>108.3254833157311</v>
+        <v>108.32548331573111</v>
       </c>
       <c r="B26">
-        <v>-12.16866787117159</v>
+        <v>-12.168667871171589</v>
       </c>
       <c r="C26">
-        <v>94.07602815655096</v>
+        <v>94.076028156550962</v>
       </c>
       <c r="D26">
-        <v>0.9625583213706062</v>
+        <v>0.96255832137060615</v>
       </c>
       <c r="E26">
-        <v>407.0467523908545</v>
+        <v>407.04675239085452</v>
       </c>
       <c r="F26">
-        <v>1.615546224293479E+23</v>
+        <v>1.6155462242934789E+23</v>
       </c>
       <c r="G26">
         <v>0</v>
       </c>
       <c r="H26">
-        <v>1.615546224293479E+23</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8">
+        <v>1.6155462242934789E+23</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>53.24279557054206</v>
+        <v>53.242795570542057</v>
       </c>
       <c r="B27">
         <v>28.65650475401446</v>
       </c>
       <c r="C27">
-        <v>67.7170040329604</v>
+        <v>67.717004032960403</v>
       </c>
       <c r="D27">
-        <v>0.9592247582713657</v>
+        <v>0.95922475827136566</v>
       </c>
       <c r="E27">
-        <v>213.8687376128107</v>
+        <v>213.86873761281069</v>
       </c>
       <c r="F27">
-        <v>5.419404682846908E+19</v>
+        <v>5.4194046828469076E+19</v>
       </c>
       <c r="G27">
         <v>0</v>
       </c>
       <c r="H27">
-        <v>5.419404682846908E+19</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8">
+        <v>5.4194046828469076E+19</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>140.8755274907737</v>
+        <v>140.87552749077369</v>
       </c>
       <c r="B28">
-        <v>87.3606939846464</v>
+        <v>87.360693984646403</v>
       </c>
       <c r="C28">
         <v>89.79592821525452</v>
       </c>
       <c r="D28">
-        <v>0.9630573819210442</v>
+        <v>0.96305738192104418</v>
       </c>
       <c r="E28">
-        <v>264.1693018757293</v>
+        <v>264.16930187572927</v>
       </c>
       <c r="F28">
-        <v>6.273388667483636E+20</v>
+        <v>6.2733886674836364E+20</v>
       </c>
       <c r="G28">
-        <v>15.98156837859196</v>
+        <v>15.981568378591961</v>
       </c>
       <c r="H28">
-        <v>6.273388667483636E+20</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8">
+        <v>6.2733886674836364E+20</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>191.6368956321309</v>
+        <v>191.63689563213089</v>
       </c>
       <c r="B29">
-        <v>93.05710004246659</v>
+        <v>93.057100042466587</v>
       </c>
       <c r="C29">
-        <v>9.119429207915353</v>
+        <v>9.1194292079153527</v>
       </c>
       <c r="D29">
-        <v>0.9578503820555412</v>
+        <v>0.95785038205554118</v>
       </c>
       <c r="E29">
-        <v>52.65027193136329</v>
+        <v>52.650271931363292</v>
       </c>
       <c r="F29">
-        <v>290397968458649.2</v>
+        <v>290397968458649.19</v>
       </c>
       <c r="G29">
         <v>12.01194443059372</v>
       </c>
       <c r="H29">
-        <v>290397968458714.9</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8">
+        <v>290397968458714.88</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>32.9832203402789</v>
+        <v>32.983220340278898</v>
       </c>
       <c r="B30">
-        <v>18.41106144952411</v>
+        <v>18.411061449524109</v>
       </c>
       <c r="C30">
-        <v>44.0230684376394</v>
+        <v>44.023068437639402</v>
       </c>
       <c r="D30">
-        <v>0.9535569068025044</v>
+        <v>0.95355690680250438</v>
       </c>
       <c r="E30">
         <v>117.6661808781088</v>
@@ -1178,18 +1194,18 @@
         <v>7.140840285290896E+16</v>
       </c>
     </row>
-    <row r="31" spans="1:8">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31">
-        <v>-30.04795470483844</v>
+        <v>-30.047954704838439</v>
       </c>
       <c r="B31">
-        <v>94.11834930209878</v>
+        <v>94.118349302098778</v>
       </c>
       <c r="C31">
-        <v>7.171305685311098</v>
+        <v>7.1713056853110979</v>
       </c>
       <c r="D31">
-        <v>0.922901337650142</v>
+        <v>0.92290133765014204</v>
       </c>
       <c r="E31">
         <v>0</v>
@@ -1201,21 +1217,21 @@
         <v>0</v>
       </c>
       <c r="H31">
-        <v>0.922901337650142</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8">
+        <v>0.92290133765014204</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>-78.41866092975312</v>
+        <v>-78.418660929753116</v>
       </c>
       <c r="B32">
-        <v>-21.76234123526426</v>
+        <v>-21.762341235264259</v>
       </c>
       <c r="C32">
-        <v>53.83975791084656</v>
+        <v>53.839757910846558</v>
       </c>
       <c r="D32">
-        <v>0.9058106059036407</v>
+        <v>0.90581060590364071</v>
       </c>
       <c r="E32">
         <v>0</v>
@@ -1227,47 +1243,47 @@
         <v>0</v>
       </c>
       <c r="H32">
-        <v>0.9058106059036407</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8">
+        <v>0.90581060590364071</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>40.65712616746993</v>
+        <v>40.657126167469933</v>
       </c>
       <c r="B33">
-        <v>52.70840637064757</v>
+        <v>52.708406370647573</v>
       </c>
       <c r="C33">
-        <v>69.37177460341995</v>
+        <v>69.371774603419951</v>
       </c>
       <c r="D33">
-        <v>0.9590542640775799</v>
+        <v>0.95905426407757988</v>
       </c>
       <c r="E33">
         <v>202.3638391314195</v>
       </c>
       <c r="F33">
-        <v>2.372430363633119E+19</v>
+        <v>2.3724303636331188E+19</v>
       </c>
       <c r="G33">
         <v>0</v>
       </c>
       <c r="H33">
-        <v>2.372430363633119E+19</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8">
+        <v>2.3724303636331188E+19</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>35.65824603317239</v>
+        <v>35.658246033172389</v>
       </c>
       <c r="B34">
-        <v>52.2685777491392</v>
+        <v>52.268577749139197</v>
       </c>
       <c r="C34">
-        <v>14.88390426204015</v>
+        <v>14.883904262040151</v>
       </c>
       <c r="D34">
-        <v>0.9120644599675635</v>
+        <v>0.91206445996756347</v>
       </c>
       <c r="E34">
         <v>0</v>
@@ -1279,47 +1295,47 @@
         <v>0</v>
       </c>
       <c r="H34">
-        <v>0.9120644599675635</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8">
+        <v>0.91206445996756347</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>-80.90656275110398</v>
+        <v>-80.906562751103976</v>
       </c>
       <c r="B35">
-        <v>-69.43870570754521</v>
+        <v>-69.438705707545211</v>
       </c>
       <c r="C35">
-        <v>71.76160959246192</v>
+        <v>71.761609592461923</v>
       </c>
       <c r="D35">
-        <v>0.944623247127382</v>
+        <v>0.94462324712738199</v>
       </c>
       <c r="E35">
-        <v>223.0062028778709</v>
+        <v>223.00620287787089</v>
       </c>
       <c r="F35">
-        <v>4.640712465512121E+18</v>
+        <v>4.6407124655121213E+18</v>
       </c>
       <c r="G35">
-        <v>0.004553370018423042</v>
+        <v>4.5533700184230419E-3</v>
       </c>
       <c r="H35">
-        <v>4.640712465512121E+18</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8">
+        <v>4.6407124655121213E+18</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>-57.3376295656435</v>
+        <v>-57.337629565643503</v>
       </c>
       <c r="B36">
-        <v>65.75550703813617</v>
+        <v>65.755507038136173</v>
       </c>
       <c r="C36">
-        <v>-2.976708928031506</v>
+        <v>-2.9767089280315062</v>
       </c>
       <c r="D36">
-        <v>0.9321102095525221</v>
+        <v>0.93211020955252211</v>
       </c>
       <c r="E36">
         <v>0</v>
@@ -1331,125 +1347,125 @@
         <v>0</v>
       </c>
       <c r="H36">
-        <v>0.9321102095525221</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8">
+        <v>0.93211020955252211</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>96.75068842927649</v>
+        <v>96.750688429276494</v>
       </c>
       <c r="B37">
-        <v>47.11758284091621</v>
+        <v>47.117582840916207</v>
       </c>
       <c r="C37">
-        <v>56.92199133635681</v>
+        <v>56.921991336356811</v>
       </c>
       <c r="D37">
-        <v>0.9596852990675112</v>
+        <v>0.95968529906751121</v>
       </c>
       <c r="E37">
-        <v>165.9674172118289</v>
+        <v>165.96741721182889</v>
       </c>
       <c r="F37">
-        <v>4.479054649916274E+18</v>
+        <v>4.4790546499162742E+18</v>
       </c>
       <c r="G37">
         <v>0</v>
       </c>
       <c r="H37">
-        <v>4.479054649916274E+18</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8">
+        <v>4.4790546499162742E+18</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>186.2392190595107</v>
       </c>
       <c r="B38">
-        <v>78.68519827181716</v>
+        <v>78.685198271817157</v>
       </c>
       <c r="C38">
         <v>-20.51751336559294</v>
       </c>
       <c r="D38">
-        <v>0.9487552909060902</v>
+        <v>0.94875529090609023</v>
       </c>
       <c r="E38">
-        <v>10.69194805595341</v>
+        <v>10.691948055953411</v>
       </c>
       <c r="F38">
-        <v>192124383997.9864</v>
+        <v>192124383997.98639</v>
       </c>
       <c r="G38">
-        <v>3.827682076206029</v>
+        <v>3.8276820762060288</v>
       </c>
       <c r="H38">
         <v>192124384013.4548</v>
       </c>
     </row>
-    <row r="39" spans="1:8">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39">
-        <v>85.03507405622499</v>
+        <v>85.035074056224985</v>
       </c>
       <c r="B39">
-        <v>53.15713797268123</v>
+        <v>53.157137972681227</v>
       </c>
       <c r="C39">
-        <v>23.36988750460016</v>
+        <v>23.369887504600161</v>
       </c>
       <c r="D39">
-        <v>0.9529435813356134</v>
+        <v>0.95294358133561341</v>
       </c>
       <c r="E39">
         <v>65.41658469644554</v>
       </c>
       <c r="F39">
-        <v>624484027318881.8</v>
+        <v>624484027318881.75</v>
       </c>
       <c r="G39">
         <v>0</v>
       </c>
       <c r="H39">
-        <v>624484027318948.1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8">
+        <v>624484027318948.13</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40">
-        <v>174.2616750625193</v>
+        <v>174.26167506251929</v>
       </c>
       <c r="B40">
-        <v>55.15056598023897</v>
+        <v>55.150565980238973</v>
       </c>
       <c r="C40">
-        <v>51.70426132469103</v>
+        <v>51.704261324691032</v>
       </c>
       <c r="D40">
-        <v>0.9614543759284989</v>
+        <v>0.96145437592849892</v>
       </c>
       <c r="E40">
-        <v>153.7068753024994</v>
+        <v>153.70687530249941</v>
       </c>
       <c r="F40">
-        <v>3.116327235054963E+18</v>
+        <v>3.1163272350549632E+18</v>
       </c>
       <c r="G40">
-        <v>9.918011155161089</v>
+        <v>9.9180111551610892</v>
       </c>
       <c r="H40">
-        <v>3.116327235054963E+18</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8">
+        <v>3.1163272350549632E+18</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>0.5415334546033379</v>
       </c>
       <c r="B41">
-        <v>-79.135912180913</v>
+        <v>-79.135912180912996</v>
       </c>
       <c r="C41">
-        <v>27.28937374444924</v>
+        <v>27.289373744449239</v>
       </c>
       <c r="D41">
-        <v>0.9113987200811153</v>
+        <v>0.91139872008111533</v>
       </c>
       <c r="E41">
         <v>0</v>
@@ -1461,38 +1477,38 @@
         <v>0</v>
       </c>
       <c r="H41">
-        <v>0.9113987200811153</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8">
+        <v>0.91139872008111533</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42">
-        <v>-25.5088442681311</v>
+        <v>-25.508844268131099</v>
       </c>
       <c r="B42">
-        <v>19.3755557316556</v>
+        <v>19.375555731655599</v>
       </c>
       <c r="C42">
-        <v>58.03460958819397</v>
+        <v>58.034609588193973</v>
       </c>
       <c r="D42">
         <v>0.9517419214834929</v>
       </c>
       <c r="E42">
-        <v>148.7983433547301</v>
+        <v>148.79834335473009</v>
       </c>
       <c r="F42">
-        <v>3.486901665315877E+17</v>
+        <v>3.4869016653158771E+17</v>
       </c>
       <c r="G42">
         <v>0</v>
       </c>
       <c r="H42">
-        <v>3.486901665315878E+17</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8">
+        <v>3.4869016653158778E+17</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43">
-        <v>-38.57723882927728</v>
+        <v>-38.577238829277277</v>
       </c>
       <c r="B43">
         <v>-79.79741907435691</v>
@@ -1501,7 +1517,7 @@
         <v>25.6192528349786</v>
       </c>
       <c r="D43">
-        <v>0.9169445831474922</v>
+        <v>0.91694458314749216</v>
       </c>
       <c r="E43">
         <v>0</v>
@@ -1510,91 +1526,91 @@
         <v>0</v>
       </c>
       <c r="G43">
-        <v>5.217834586475211</v>
+        <v>5.2178345864752114</v>
       </c>
       <c r="H43">
-        <v>6.134779169622703</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8">
+        <v>6.1347791696227034</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44">
-        <v>-14.98159267416806</v>
+        <v>-14.981592674168059</v>
       </c>
       <c r="B44">
-        <v>-69.48695555595729</v>
+        <v>-69.486955555957294</v>
       </c>
       <c r="C44">
-        <v>75.54336847712315</v>
+        <v>75.543368477123153</v>
       </c>
       <c r="D44">
-        <v>0.9564241603024884</v>
+        <v>0.95642416030248845</v>
       </c>
       <c r="E44">
-        <v>342.9965182825895</v>
+        <v>342.99651828258948</v>
       </c>
       <c r="F44">
-        <v>8.68657903658135E+21</v>
+        <v>8.6865790365813503E+21</v>
       </c>
       <c r="G44">
         <v>0</v>
       </c>
       <c r="H44">
-        <v>8.68657903658135E+21</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8">
+        <v>8.6865790365813503E+21</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>-50.65199822140098</v>
       </c>
       <c r="B45">
-        <v>69.49585727714444</v>
+        <v>69.495857277144438</v>
       </c>
       <c r="C45">
-        <v>84.31118698812298</v>
+        <v>84.311186988122984</v>
       </c>
       <c r="D45">
-        <v>0.9570715156144429</v>
+        <v>0.95707151561444292</v>
       </c>
       <c r="E45">
         <v>244.254128248413</v>
       </c>
       <c r="F45">
-        <v>7.733025424556715E+19</v>
+        <v>7.7330254245567152E+19</v>
       </c>
       <c r="G45">
         <v>0</v>
       </c>
       <c r="H45">
-        <v>7.733025424556715E+19</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8">
+        <v>7.7330254245567152E+19</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46">
-        <v>21.02753001507027</v>
+        <v>21.027530015070269</v>
       </c>
       <c r="B46">
-        <v>4.108688315749864</v>
+        <v>4.1086883157498644</v>
       </c>
       <c r="C46">
-        <v>84.05053539069499</v>
+        <v>84.050535390694989</v>
       </c>
       <c r="D46">
         <v>0.9597402661515757</v>
       </c>
       <c r="E46">
-        <v>322.1102133999772</v>
+        <v>322.11021339997723</v>
       </c>
       <c r="F46">
-        <v>5.308433028579776E+21</v>
+        <v>5.3084330285797757E+21</v>
       </c>
       <c r="G46">
         <v>0</v>
       </c>
       <c r="H46">
-        <v>5.308433028579776E+21</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8">
+        <v>5.3084330285797757E+21</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>122.5781728859378</v>
       </c>
@@ -1611,7 +1627,7 @@
         <v>0</v>
       </c>
       <c r="F47">
-        <v>10187774.40480353</v>
+        <v>10187774.404803529</v>
       </c>
       <c r="G47">
         <v>0</v>
@@ -1620,73 +1636,73 @@
         <v>10187775.32961574</v>
       </c>
     </row>
-    <row r="48" spans="1:8">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48">
-        <v>39.1729550954119</v>
+        <v>39.172955095411901</v>
       </c>
       <c r="B48">
-        <v>-52.98248213987991</v>
+        <v>-52.982482139879913</v>
       </c>
       <c r="C48">
-        <v>67.63792716401423</v>
+        <v>67.637927164014229</v>
       </c>
       <c r="D48">
         <v>0.9581841050714992</v>
       </c>
       <c r="E48">
-        <v>282.0420125675407</v>
+        <v>282.04201256754072</v>
       </c>
       <c r="F48">
-        <v>1.568380083466476E+21</v>
+        <v>1.5683800834664759E+21</v>
       </c>
       <c r="G48">
         <v>0</v>
       </c>
       <c r="H48">
-        <v>1.568380083466476E+21</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8">
+        <v>1.5683800834664759E+21</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49">
-        <v>8.503012391985182</v>
+        <v>8.5030123919851821</v>
       </c>
       <c r="B49">
-        <v>1.214075573120914</v>
+        <v>1.2140755731209141</v>
       </c>
       <c r="C49">
-        <v>68.01084899033417</v>
+        <v>68.010848990334168</v>
       </c>
       <c r="D49">
-        <v>0.9570517143115491</v>
+        <v>0.95705171431154912</v>
       </c>
       <c r="E49">
-        <v>226.3210104870171</v>
+        <v>226.32101048701711</v>
       </c>
       <c r="F49">
-        <v>7.150657648244398E+19</v>
+        <v>7.1506576482443977E+19</v>
       </c>
       <c r="G49">
         <v>0</v>
       </c>
       <c r="H49">
-        <v>7.150657648244398E+19</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8">
+        <v>7.1506576482443977E+19</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>48.89408446979029</v>
+        <v>48.894084469790293</v>
       </c>
       <c r="B50">
-        <v>18.87072216233638</v>
+        <v>18.870722162336381</v>
       </c>
       <c r="C50">
-        <v>70.46545388749948</v>
+        <v>70.465453887499478</v>
       </c>
       <c r="D50">
         <v>0.9593286288341154</v>
       </c>
       <c r="E50">
-        <v>233.6749495187805</v>
+        <v>233.67494951878049</v>
       </c>
       <c r="F50">
         <v>1.481852477508277E+20</v>
@@ -1698,15 +1714,15 @@
         <v>1.481852477508277E+20</v>
       </c>
     </row>
-    <row r="51" spans="1:8">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>-65.56745386324741</v>
+        <v>-65.567453863247408</v>
       </c>
       <c r="B51">
-        <v>73.19909988402043</v>
+        <v>73.199099884020427</v>
       </c>
       <c r="C51">
-        <v>26.42310724727349</v>
+        <v>26.423107247273489</v>
       </c>
       <c r="D51">
         <v>0.9173424061918044</v>
@@ -1724,18 +1740,18 @@
         <v>0.9173424061918044</v>
       </c>
     </row>
-    <row r="52" spans="1:8">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52">
-        <v>-11.55236965433208</v>
+        <v>-11.552369654332081</v>
       </c>
       <c r="B52">
-        <v>27.47885480046221</v>
+        <v>27.478854800462209</v>
       </c>
       <c r="C52">
-        <v>3.707653028146103</v>
+        <v>3.7076530281461029</v>
       </c>
       <c r="D52">
-        <v>0.9236206137030447</v>
+        <v>0.92362061370304471</v>
       </c>
       <c r="E52">
         <v>0</v>
@@ -1747,12 +1763,12 @@
         <v>0</v>
       </c>
       <c r="H52">
-        <v>0.9236206137030447</v>
-      </c>
-    </row>
-    <row r="53" spans="1:8">
+        <v>0.92362061370304471</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53">
-        <v>-51.85643440045509</v>
+        <v>-51.856434400455093</v>
       </c>
       <c r="B53">
         <v>-42</v>
@@ -1761,7 +1777,7 @@
         <v>24</v>
       </c>
       <c r="D53">
-        <v>0.9188052932341206</v>
+        <v>0.91880529323412063</v>
       </c>
       <c r="E53">
         <v>0</v>
@@ -1773,10 +1789,10 @@
         <v>0</v>
       </c>
       <c r="H53">
-        <v>0.9188052932341206</v>
-      </c>
-    </row>
-    <row r="54" spans="1:8">
+        <v>0.91880529323412063</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>147.557720340922</v>
       </c>
@@ -1784,13 +1800,13 @@
         <v>14.94310975404572</v>
       </c>
       <c r="C54">
-        <v>17.32143581736595</v>
+        <v>17.321435817365948</v>
       </c>
       <c r="D54">
-        <v>0.9561914343385975</v>
+        <v>0.95619143433859755</v>
       </c>
       <c r="E54">
-        <v>74.55573158323814</v>
+        <v>74.555731583238142</v>
       </c>
       <c r="F54">
         <v>3942033669005224</v>
@@ -1802,18 +1818,18 @@
         <v>3942033669005300</v>
       </c>
     </row>
-    <row r="55" spans="1:8">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55">
-        <v>-47.31107251820578</v>
+        <v>-47.311072518205783</v>
       </c>
       <c r="B55">
-        <v>-33.96776612868369</v>
+        <v>-33.967766128683692</v>
       </c>
       <c r="C55">
-        <v>-19.02145846217092</v>
+        <v>-19.021458462170919</v>
       </c>
       <c r="D55">
-        <v>0.9416528864928848</v>
+        <v>0.94165288649288481</v>
       </c>
       <c r="E55">
         <v>0</v>
@@ -1822,27 +1838,27 @@
         <v>0</v>
       </c>
       <c r="G55">
-        <v>8.451921285114029</v>
+        <v>8.4519212851140288</v>
       </c>
       <c r="H55">
-        <v>9.393574171606915</v>
-      </c>
-    </row>
-    <row r="56" spans="1:8">
+        <v>9.3935741716069145</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>162.9913923502757</v>
       </c>
       <c r="B56">
-        <v>-19.76931042829912</v>
+        <v>-19.769310428299121</v>
       </c>
       <c r="C56">
-        <v>94.07602815655096</v>
+        <v>94.076028156550962</v>
       </c>
       <c r="D56">
-        <v>0.9634228121866049</v>
+        <v>0.96342281218660486</v>
       </c>
       <c r="E56">
-        <v>407.3351093896965</v>
+        <v>407.33510938969653</v>
       </c>
       <c r="F56">
         <v>1.976755079950715E+23</v>
@@ -1854,70 +1870,70 @@
         <v>1.976755079950715E+23</v>
       </c>
     </row>
-    <row r="57" spans="1:8">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57">
-        <v>93.91312321266089</v>
+        <v>93.913123212660892</v>
       </c>
       <c r="B57">
-        <v>-2.865097717563334</v>
+        <v>-2.8650977175633341</v>
       </c>
       <c r="C57">
-        <v>63.55570547563907</v>
+        <v>63.555705475639073</v>
       </c>
       <c r="D57">
-        <v>0.960055873964525</v>
+        <v>0.96005587396452496</v>
       </c>
       <c r="E57">
-        <v>224.1829639993044</v>
+        <v>224.18296399930441</v>
       </c>
       <c r="F57">
-        <v>1.478941703514685E+20</v>
+        <v>1.4789417035146851E+20</v>
       </c>
       <c r="G57">
         <v>0</v>
       </c>
       <c r="H57">
-        <v>1.478941703514685E+20</v>
-      </c>
-    </row>
-    <row r="58" spans="1:8">
+        <v>1.4789417035146851E+20</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58">
-        <v>140.8755274907737</v>
+        <v>140.87552749077369</v>
       </c>
       <c r="B58">
-        <v>45.75638980789272</v>
+        <v>45.756389807892717</v>
       </c>
       <c r="C58">
-        <v>66.76566599242786</v>
+        <v>66.765665992427856</v>
       </c>
       <c r="D58">
-        <v>0.9617027813827652</v>
+        <v>0.96170278138276521</v>
       </c>
       <c r="E58">
-        <v>206.2167146679413</v>
+        <v>206.21671466794129</v>
       </c>
       <c r="F58">
-        <v>5.877235736184354E+19</v>
+        <v>5.8772357361843544E+19</v>
       </c>
       <c r="G58">
-        <v>5.323149238828351</v>
+        <v>5.3231492388283508</v>
       </c>
       <c r="H58">
-        <v>5.877235736184354E+19</v>
-      </c>
-    </row>
-    <row r="59" spans="1:8">
+        <v>5.8772357361843544E+19</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>-62.80866992331169</v>
       </c>
       <c r="B59">
-        <v>-69.85326539075454</v>
+        <v>-69.853265390754544</v>
       </c>
       <c r="C59">
-        <v>9.119429207915353</v>
+        <v>9.1194292079153527</v>
       </c>
       <c r="D59">
-        <v>0.9287457431770089</v>
+        <v>0.92874574317700886</v>
       </c>
       <c r="E59">
         <v>0</v>
@@ -1926,79 +1942,79 @@
         <v>0</v>
       </c>
       <c r="G59">
-        <v>21.14432192276716</v>
+        <v>21.144321922767158</v>
       </c>
       <c r="H59">
-        <v>22.07306766594417</v>
-      </c>
-    </row>
-    <row r="60" spans="1:8">
+        <v>22.073067665944169</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>118.560018098562</v>
       </c>
       <c r="B60">
-        <v>17.48275208322435</v>
+        <v>17.482752083224351</v>
       </c>
       <c r="C60">
-        <v>63.22772023642793</v>
+        <v>63.227720236427928</v>
       </c>
       <c r="D60">
-        <v>0.960820639284739</v>
+        <v>0.96082063928473904</v>
       </c>
       <c r="E60">
-        <v>210.3428967150998</v>
+        <v>210.34289671509981</v>
       </c>
       <c r="F60">
-        <v>7.71111986497451E+19</v>
+        <v>7.7111198649745097E+19</v>
       </c>
       <c r="G60">
         <v>0</v>
       </c>
       <c r="H60">
-        <v>7.71111986497451E+19</v>
-      </c>
-    </row>
-    <row r="61" spans="1:8">
+        <v>7.7111198649745097E+19</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61">
-        <v>-30.04795470483844</v>
+        <v>-30.047954704838439</v>
       </c>
       <c r="B61">
-        <v>-51.40957827127009</v>
+        <v>-51.409578271270092</v>
       </c>
       <c r="C61">
-        <v>95.48242753268622</v>
+        <v>95.482427532686216</v>
       </c>
       <c r="D61">
-        <v>0.9588825219877575</v>
+        <v>0.95888252198775747</v>
       </c>
       <c r="E61">
-        <v>507.4453781196979</v>
+        <v>507.44537811969792</v>
       </c>
       <c r="F61">
-        <v>1.096355644399974E+24</v>
+        <v>1.0963556443999741E+24</v>
       </c>
       <c r="G61">
         <v>0</v>
       </c>
       <c r="H61">
-        <v>1.096355644399974E+24</v>
-      </c>
-    </row>
-    <row r="62" spans="1:8">
+        <v>1.0963556443999741E+24</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62">
-        <v>-78.41866092975312</v>
+        <v>-78.418660929753116</v>
       </c>
       <c r="B62">
-        <v>-55.18682829596108</v>
+        <v>-55.186828295961078</v>
       </c>
       <c r="C62">
-        <v>91.36054561437632</v>
+        <v>91.360545614376321</v>
       </c>
       <c r="D62">
-        <v>0.9555361943529466</v>
+        <v>0.95553619435294657</v>
       </c>
       <c r="E62">
-        <v>450.1820865665782</v>
+        <v>450.18208656657822</v>
       </c>
       <c r="F62">
         <v>1.063516747405638E+23</v>
@@ -2010,15 +2026,15 @@
         <v>1.063516747405638E+23</v>
       </c>
     </row>
-    <row r="63" spans="1:8">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63">
-        <v>-70.32262776560982</v>
+        <v>-70.322627765609823</v>
       </c>
       <c r="B63">
         <v>3.02804304071238</v>
       </c>
       <c r="C63">
-        <v>38.29295578303363</v>
+        <v>38.292955783033626</v>
       </c>
       <c r="D63">
         <v>0.9126947296230824</v>
@@ -2036,73 +2052,73 @@
         <v>0.9126947296230824</v>
       </c>
     </row>
-    <row r="64" spans="1:8">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64">
-        <v>35.65824603317239</v>
+        <v>35.658246033172389</v>
       </c>
       <c r="B64">
-        <v>60.52367825530901</v>
+        <v>60.523678255309008</v>
       </c>
       <c r="C64">
-        <v>71.34279302375933</v>
+        <v>71.342793023759327</v>
       </c>
       <c r="D64">
-        <v>0.9591314094574457</v>
+        <v>0.95913140945744568</v>
       </c>
       <c r="E64">
         <v>204.722145318006</v>
       </c>
       <c r="F64">
-        <v>2.500818889000463E+19</v>
+        <v>2.5008188890004632E+19</v>
       </c>
       <c r="G64">
         <v>0</v>
       </c>
       <c r="H64">
-        <v>2.500818889000463E+19</v>
-      </c>
-    </row>
-    <row r="65" spans="1:8">
+        <v>2.5008188890004632E+19</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65">
-        <v>-37.33542409818224</v>
+        <v>-37.335424098182237</v>
       </c>
       <c r="B65">
-        <v>0.4660181440162572</v>
+        <v>0.46601814401625719</v>
       </c>
       <c r="C65">
-        <v>87.44041778105739</v>
+        <v>87.440417781057391</v>
       </c>
       <c r="D65">
-        <v>0.9577697446679327</v>
+        <v>0.95776974466793274</v>
       </c>
       <c r="E65">
-        <v>341.5559619211754</v>
+        <v>341.55596192117542</v>
       </c>
       <c r="F65">
-        <v>5.928104032434503E+21</v>
+        <v>5.9281040324345033E+21</v>
       </c>
       <c r="G65">
         <v>0</v>
       </c>
       <c r="H65">
-        <v>5.928104032434503E+21</v>
-      </c>
-    </row>
-    <row r="66" spans="1:8">
+        <v>5.9281040324345033E+21</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>25.86515104152798</v>
       </c>
       <c r="B66">
-        <v>-4.07496321896193</v>
+        <v>-4.0749632189619298</v>
       </c>
       <c r="C66">
-        <v>69.32570283720466</v>
+        <v>69.325702837204659</v>
       </c>
       <c r="D66">
-        <v>0.9581106301901007</v>
+        <v>0.95811063019010068</v>
       </c>
       <c r="E66">
-        <v>242.5502733951517</v>
+        <v>242.55027339515169</v>
       </c>
       <c r="F66">
         <v>1.983222525186879E+20</v>
@@ -2114,44 +2130,44 @@
         <v>1.983222525186879E+20</v>
       </c>
     </row>
-    <row r="67" spans="1:8">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>-74.82429104730808</v>
       </c>
       <c r="B67">
-        <v>-44.55292721182958</v>
+        <v>-44.552927211829576</v>
       </c>
       <c r="C67">
-        <v>76.31152858603902</v>
+        <v>76.311528586039017</v>
       </c>
       <c r="D67">
         <v>0.9511890094859804</v>
       </c>
       <c r="E67">
-        <v>275.1211569532657</v>
+        <v>275.12115695326571</v>
       </c>
       <c r="F67">
-        <v>1.627601804974983E+20</v>
+        <v>1.6276018049749831E+20</v>
       </c>
       <c r="G67">
         <v>0</v>
       </c>
       <c r="H67">
-        <v>1.627601804974983E+20</v>
-      </c>
-    </row>
-    <row r="68" spans="1:8">
+        <v>1.6276018049749831E+20</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68">
-        <v>-81.83765998490031</v>
+        <v>-81.837659984900313</v>
       </c>
       <c r="B68">
-        <v>-29.86465170958103</v>
+        <v>-29.864651709581029</v>
       </c>
       <c r="C68">
         <v>-20.51751336559294</v>
       </c>
       <c r="D68">
-        <v>0.9468905081232596</v>
+        <v>0.94689050812325959</v>
       </c>
       <c r="E68">
         <v>0</v>
@@ -2160,24 +2176,24 @@
         <v>0</v>
       </c>
       <c r="G68">
-        <v>27.29122571660401</v>
+        <v>27.291225716604011</v>
       </c>
       <c r="H68">
-        <v>28.23811622472727</v>
-      </c>
-    </row>
-    <row r="69" spans="1:8">
+        <v>28.238116224727271</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69">
-        <v>-80.64371481221453</v>
+        <v>-80.643714812214526</v>
       </c>
       <c r="B69">
         <v>-26.76931756550902</v>
       </c>
       <c r="C69">
-        <v>56.58943292175474</v>
+        <v>56.589432921754742</v>
       </c>
       <c r="D69">
-        <v>0.904695240648448</v>
+        <v>0.90469524064844797</v>
       </c>
       <c r="E69">
         <v>0</v>
@@ -2189,73 +2205,73 @@
         <v>0</v>
       </c>
       <c r="H69">
-        <v>0.904695240648448</v>
-      </c>
-    </row>
-    <row r="70" spans="1:8">
+        <v>0.90469524064844797</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>158.8437365647612</v>
       </c>
       <c r="B70">
-        <v>-7.833215800789361</v>
+        <v>-7.8332158007893611</v>
       </c>
       <c r="C70">
-        <v>63.07403750835461</v>
+        <v>63.074037508354607</v>
       </c>
       <c r="D70">
-        <v>0.961725055237472</v>
+        <v>0.96172505523747198</v>
       </c>
       <c r="E70">
-        <v>231.2384842725801</v>
+        <v>231.23848427258011</v>
       </c>
       <c r="F70">
-        <v>3.18940012876531E+20</v>
+        <v>3.1894001287653097E+20</v>
       </c>
       <c r="G70">
         <v>0</v>
       </c>
       <c r="H70">
-        <v>3.18940012876531E+20</v>
-      </c>
-    </row>
-    <row r="71" spans="1:8">
+        <v>3.1894001287653097E+20</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>0.5415334546033379</v>
       </c>
       <c r="B71">
-        <v>-79.135912180913</v>
+        <v>-79.135912180912996</v>
       </c>
       <c r="C71">
-        <v>56.65578921025947</v>
+        <v>56.655789210259471</v>
       </c>
       <c r="D71">
-        <v>0.9525250375417154</v>
+        <v>0.95252503754171536</v>
       </c>
       <c r="E71">
         <v>211.1347942760018</v>
       </c>
       <c r="F71">
-        <v>2.368458457140998E+19</v>
+        <v>2.3684584571409981E+19</v>
       </c>
       <c r="G71">
         <v>0</v>
       </c>
       <c r="H71">
-        <v>2.368458457140998E+19</v>
-      </c>
-    </row>
-    <row r="72" spans="1:8">
+        <v>2.3684584571409981E+19</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72">
-        <v>-22.70191874311738</v>
+        <v>-22.701918743117378</v>
       </c>
       <c r="B72">
-        <v>-64.5094612953675</v>
+        <v>-64.509461295367501</v>
       </c>
       <c r="C72">
         <v>-4.450979240034818</v>
       </c>
       <c r="D72">
-        <v>0.9310832702502042</v>
+        <v>0.93108327025020421</v>
       </c>
       <c r="E72">
         <v>0</v>
@@ -2264,53 +2280,53 @@
         <v>0</v>
       </c>
       <c r="G72">
-        <v>4.77798220416199</v>
+        <v>4.7779822041619902</v>
       </c>
       <c r="H72">
-        <v>5.709065474412195</v>
-      </c>
-    </row>
-    <row r="73" spans="1:8">
+        <v>5.7090654744121947</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73">
-        <v>130.2662164633718</v>
+        <v>130.26621646337179</v>
       </c>
       <c r="B73">
-        <v>-30.55312971978453</v>
+        <v>-30.553129719784529</v>
       </c>
       <c r="C73">
-        <v>47.45090295253222</v>
+        <v>47.450902952532218</v>
       </c>
       <c r="D73">
-        <v>0.959510690958542</v>
+        <v>0.95951069095854202</v>
       </c>
       <c r="E73">
-        <v>179.5300783701721</v>
+        <v>179.53007837017211</v>
       </c>
       <c r="F73">
-        <v>1.963840217376257E+19</v>
+        <v>1.9638402173762568E+19</v>
       </c>
       <c r="G73">
         <v>0</v>
       </c>
       <c r="H73">
-        <v>1.963840217376257E+19</v>
-      </c>
-    </row>
-    <row r="74" spans="1:8">
+        <v>1.9638402173762568E+19</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74">
-        <v>188.6425809391227</v>
+        <v>188.64258093912269</v>
       </c>
       <c r="B74">
-        <v>-45.36360340834702</v>
+        <v>-45.363603408347018</v>
       </c>
       <c r="C74">
-        <v>9.055684584822078</v>
+        <v>9.0556845848220782</v>
       </c>
       <c r="D74">
-        <v>0.95666453659402</v>
+        <v>0.95666453659401995</v>
       </c>
       <c r="E74">
-        <v>77.60130483572721</v>
+        <v>77.601304835727206</v>
       </c>
       <c r="F74">
         <v>9996488397646218</v>
@@ -2322,44 +2338,44 @@
         <v>9996488397646296</v>
       </c>
     </row>
-    <row r="75" spans="1:8">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75">
-        <v>10.76306387382449</v>
+        <v>10.763063873824491</v>
       </c>
       <c r="B75">
-        <v>81.68631743605252</v>
+        <v>81.686317436052519</v>
       </c>
       <c r="C75">
-        <v>58.8722268261146</v>
+        <v>58.872226826114598</v>
       </c>
       <c r="D75">
-        <v>0.9561818505081194</v>
+        <v>0.95618185050811944</v>
       </c>
       <c r="E75">
-        <v>139.7887746719277</v>
+        <v>139.78877467192771</v>
       </c>
       <c r="F75">
-        <v>3.045518350591146E+17</v>
+        <v>3.0455183505911462E+17</v>
       </c>
       <c r="G75">
         <v>0</v>
       </c>
       <c r="H75">
-        <v>3.045518350591147E+17</v>
-      </c>
-    </row>
-    <row r="76" spans="1:8">
+        <v>3.0455183505911469E+17</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76">
-        <v>-40.64768785760109</v>
+        <v>-40.647687857601092</v>
       </c>
       <c r="B76">
-        <v>-38.39414880939423</v>
+        <v>-38.394148809394231</v>
       </c>
       <c r="C76">
-        <v>43.24282330125354</v>
+        <v>43.242823301253537</v>
       </c>
       <c r="D76">
-        <v>0.9072324688591074</v>
+        <v>0.90723246885910735</v>
       </c>
       <c r="E76">
         <v>0</v>
@@ -2371,10 +2387,10 @@
         <v>0</v>
       </c>
       <c r="H76">
-        <v>0.9072324688591074</v>
-      </c>
-    </row>
-    <row r="77" spans="1:8">
+        <v>0.90723246885910735</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>-10.33214206541636</v>
       </c>
@@ -2385,7 +2401,7 @@
         <v>34.12115949719206</v>
       </c>
       <c r="D77">
-        <v>0.9078400823706568</v>
+        <v>0.90784008237065683</v>
       </c>
       <c r="E77">
         <v>0</v>
@@ -2397,47 +2413,47 @@
         <v>0</v>
       </c>
       <c r="H77">
-        <v>0.9078400823706568</v>
-      </c>
-    </row>
-    <row r="78" spans="1:8">
+        <v>0.90784008237065683</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>36.67454132776642</v>
       </c>
       <c r="B78">
-        <v>-30.3352964624189</v>
+        <v>-30.335296462418899</v>
       </c>
       <c r="C78">
-        <v>39.09730158240382</v>
+        <v>39.097301582403823</v>
       </c>
       <c r="D78">
-        <v>0.9511451003469396</v>
+        <v>0.95114510034693955</v>
       </c>
       <c r="E78">
         <v>114.9223080866017</v>
       </c>
       <c r="F78">
-        <v>5.248842434061571E+16</v>
+        <v>5.2488424340615712E+16</v>
       </c>
       <c r="G78">
         <v>0</v>
       </c>
       <c r="H78">
-        <v>5.248842434061582E+16</v>
-      </c>
-    </row>
-    <row r="79" spans="1:8">
+        <v>5.2488424340615824E+16</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79">
-        <v>-5.984719381434711</v>
+        <v>-5.9847193814347106</v>
       </c>
       <c r="B79">
-        <v>-53.80456566350353</v>
+        <v>-53.804565663503531</v>
       </c>
       <c r="C79">
-        <v>10.80271654993171</v>
+        <v>10.802716549931709</v>
       </c>
       <c r="D79">
-        <v>0.9205450288981318</v>
+        <v>0.92054502889813183</v>
       </c>
       <c r="E79">
         <v>0</v>
@@ -2449,24 +2465,24 @@
         <v>0</v>
       </c>
       <c r="H79">
-        <v>0.9205450288981318</v>
-      </c>
-    </row>
-    <row r="80" spans="1:8">
+        <v>0.92054502889813183</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>171.0101751860725</v>
       </c>
       <c r="B80">
-        <v>-74.90424875597331</v>
+        <v>-74.904248755973313</v>
       </c>
       <c r="C80">
-        <v>70.46545388749948</v>
+        <v>70.465453887499478</v>
       </c>
       <c r="D80">
-        <v>0.9622854190960112</v>
+        <v>0.96228541909601117</v>
       </c>
       <c r="E80">
-        <v>336.1449905285577</v>
+        <v>336.14499052855768</v>
       </c>
       <c r="F80">
         <v>3.593544588148865E+22</v>
@@ -2478,96 +2494,96 @@
         <v>3.593544588148865E+22</v>
       </c>
     </row>
-    <row r="81" spans="1:8">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81">
-        <v>176.0547201602122</v>
+        <v>176.05472016021221</v>
       </c>
       <c r="B81">
         <v>-16.72100047554131</v>
       </c>
       <c r="C81">
-        <v>26.42310724727349</v>
+        <v>26.423107247273489</v>
       </c>
       <c r="D81">
-        <v>0.958878249643621</v>
+        <v>0.95887824964362101</v>
       </c>
       <c r="E81">
-        <v>111.6748808882977</v>
+        <v>111.67488088829769</v>
       </c>
       <c r="F81">
-        <v>2.125791396674842E+17</v>
+        <v>2.1257913966748419E+17</v>
       </c>
       <c r="G81">
         <v>0</v>
       </c>
       <c r="H81">
-        <v>2.125791396674844E+17</v>
-      </c>
-    </row>
-    <row r="82" spans="1:8">
+        <v>2.1257913966748442E+17</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82">
-        <v>-23.49007972685775</v>
+        <v>-23.490079726857751</v>
       </c>
       <c r="B82">
-        <v>27.47885480046221</v>
+        <v>27.478854800462209</v>
       </c>
       <c r="C82">
-        <v>87.97763214319453</v>
+        <v>87.977632143194526</v>
       </c>
       <c r="D82">
-        <v>0.9586355484354824</v>
+        <v>0.95863554843548238</v>
       </c>
       <c r="E82">
-        <v>314.6683053870885</v>
+        <v>314.66830538708848</v>
       </c>
       <c r="F82">
-        <v>2.388769723252684E+21</v>
+        <v>2.3887697232526841E+21</v>
       </c>
       <c r="G82">
         <v>0</v>
       </c>
       <c r="H82">
-        <v>2.388769723252684E+21</v>
-      </c>
-    </row>
-    <row r="83" spans="1:8">
+        <v>2.3887697232526841E+21</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83">
-        <v>-56.48801412409185</v>
+        <v>-56.488014124091848</v>
       </c>
       <c r="B83">
         <v>-42</v>
       </c>
       <c r="C83">
-        <v>62.30785399484956</v>
+        <v>62.307853994849559</v>
       </c>
       <c r="D83">
-        <v>0.9449220580432847</v>
+        <v>0.94492205804328466</v>
       </c>
       <c r="E83">
-        <v>163.7963959100229</v>
+        <v>163.79639591002291</v>
       </c>
       <c r="F83">
-        <v>2.687527127155586E+17</v>
+        <v>2.6875271271555859E+17</v>
       </c>
       <c r="G83">
         <v>0</v>
       </c>
       <c r="H83">
-        <v>2.687527127155588E+17</v>
-      </c>
-    </row>
-    <row r="84" spans="1:8">
+        <v>2.6875271271555878E+17</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84">
-        <v>-89.64099453785457</v>
+        <v>-89.640994537854567</v>
       </c>
       <c r="B84">
         <v>-14.68800577598072</v>
       </c>
       <c r="C84">
-        <v>29.55694190448853</v>
+        <v>29.556941904488529</v>
       </c>
       <c r="D84">
-        <v>0.9199367430733075</v>
+        <v>0.91993674307330753</v>
       </c>
       <c r="E84">
         <v>0</v>
@@ -2579,18 +2595,18 @@
         <v>0</v>
       </c>
       <c r="H84">
-        <v>0.9199367430733075</v>
-      </c>
-    </row>
-    <row r="85" spans="1:8">
+        <v>0.91993674307330753</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85">
-        <v>-47.31107251820578</v>
+        <v>-47.311072518205783</v>
       </c>
       <c r="B85">
-        <v>-33.96776612868369</v>
+        <v>-33.967766128683692</v>
       </c>
       <c r="C85">
-        <v>73.26408492087953</v>
+        <v>73.264084920879526</v>
       </c>
       <c r="D85">
         <v>0.9536845464585324</v>
@@ -2608,15 +2624,15 @@
         <v>1.962004568726431E+20</v>
       </c>
     </row>
-    <row r="86" spans="1:8">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86">
-        <v>51.85796895134666</v>
+        <v>51.857968951346663</v>
       </c>
       <c r="B86">
-        <v>-51.52930237838071</v>
+        <v>-51.529302378380713</v>
       </c>
       <c r="C86">
-        <v>41.62994210137989</v>
+        <v>41.629942101379889</v>
       </c>
       <c r="D86">
         <v>0.9536305506263999</v>
@@ -2625,27 +2641,27 @@
         <v>142.5225936349045</v>
       </c>
       <c r="F86">
-        <v>6.770397766987084E+17</v>
+        <v>6.7703977669870835E+17</v>
       </c>
       <c r="G86">
         <v>0</v>
       </c>
       <c r="H86">
-        <v>6.770397766987085E+17</v>
-      </c>
-    </row>
-    <row r="87" spans="1:8">
+        <v>6.7703977669870848E+17</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87">
-        <v>-61.13366379856975</v>
+        <v>-61.133663798569749</v>
       </c>
       <c r="B87">
         <v>28.65650475401446</v>
       </c>
       <c r="C87">
-        <v>62.52120311424511</v>
+        <v>62.521203114245111</v>
       </c>
       <c r="D87">
-        <v>0.9480118592763185</v>
+        <v>0.94801185927631848</v>
       </c>
       <c r="E87">
         <v>141.5355461890191</v>
@@ -2657,24 +2673,24 @@
         <v>0</v>
       </c>
       <c r="H87">
-        <v>9.630573769222614E+16</v>
-      </c>
-    </row>
-    <row r="88" spans="1:8">
+        <v>9.6305737692226144E+16</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88">
-        <v>-24.77288669812659</v>
+        <v>-24.772886698126591</v>
       </c>
       <c r="B88">
-        <v>90.9969292429091</v>
+        <v>90.996929242909104</v>
       </c>
       <c r="C88">
-        <v>66.76566599242786</v>
+        <v>66.765665992427856</v>
       </c>
       <c r="D88">
-        <v>0.9555077656592786</v>
+        <v>0.95550776565927864</v>
       </c>
       <c r="E88">
-        <v>155.1934333422116</v>
+        <v>155.19343334221159</v>
       </c>
       <c r="F88">
         <v>6.054361387606176E+17</v>
@@ -2683,7 +2699,7 @@
         <v>0</v>
       </c>
       <c r="H88">
-        <v>6.054361387606177E+17</v>
+        <v>6.0543613876061773E+17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>